<commit_message>
download_etf_data saves end-of-month prices to Excel file
</commit_message>
<xml_diff>
--- a/src/Risk_Parity/ETF.xlsx
+++ b/src/Risk_Parity/ETF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bfraenkel/Documents/Code/Financial_Plan/src/Risk_Parity/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103E1DC5-E6D4-D84A-9F0E-9EC02DAB1864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF34FD7C-F3A8-A342-B3CC-D81EF36DA878}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6780" yWindow="3800" windowWidth="26440" windowHeight="15440" xr2:uid="{1AC87585-0C3E-F841-A0E9-CB7E49289A23}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Ticker</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>VEMAX</t>
+  </si>
+  <si>
+    <t>VEUSX</t>
   </si>
 </sst>
 </file>
@@ -428,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C73C3887-7FFF-AE4E-A85D-C921BE7A41F0}">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
@@ -461,6 +464,11 @@
         <v>5</v>
       </c>
     </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>